<commit_message>
examples for all models
</commit_message>
<xml_diff>
--- a/examples/output/MNL_modeChoice_RP.xlsx
+++ b/examples/output/MNL_modeChoice_RP.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="30">
   <si>
     <t>Parameter</t>
   </si>
@@ -94,7 +94,13 @@
     <t>Converged</t>
   </si>
   <si>
-    <t>Estimation time (s)</t>
+    <t>Hessian at optimum</t>
+  </si>
+  <si>
+    <t>pos. def.</t>
+  </si>
+  <si>
+    <t>Estimation time (seconds)</t>
   </si>
   <si>
     <t>Number of free parameters</t>
@@ -109,7 +115,7 @@
     <t>BIC</t>
   </si>
   <si>
-    <t>Rho-squared</t>
+    <t>Rho-squared (McFadden)</t>
   </si>
 </sst>
 </file>
@@ -495,25 +501,25 @@
         <v>8</v>
       </c>
       <c r="B2">
-        <v>1.629073210400393</v>
+        <v>1.6290732103990277</v>
       </c>
       <c r="C2">
-        <v>0.8274352503686208</v>
+        <v>0.8274352503686759</v>
       </c>
       <c r="D2">
-        <v>1.968822587235248</v>
+        <v>1.9688225872334666</v>
       </c>
       <c r="E2">
-        <v>0.04897346757273602</v>
+        <v>0.04897346757294074</v>
       </c>
       <c r="F2">
-        <v>0.8141056659851807</v>
+        <v>0.8141056659852932</v>
       </c>
       <c r="G2">
-        <v>2.0010586812818563</v>
+        <v>2.0010586812799027</v>
       </c>
       <c r="H2">
-        <v>0.04538606640783627</v>
+        <v>0.045386066408046766</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -521,25 +527,25 @@
         <v>9</v>
       </c>
       <c r="B3">
-        <v>0.47467669268731216</v>
+        <v>0.4746766926866607</v>
       </c>
       <c r="C3">
-        <v>1.0186722165192739</v>
+        <v>1.01867221651924</v>
       </c>
       <c r="D3">
-        <v>0.4659758899769021</v>
+        <v>0.4659758899762781</v>
       </c>
       <c r="E3">
-        <v>0.6412327583488708</v>
+        <v>0.6412327583493174</v>
       </c>
       <c r="F3">
-        <v>0.9916823152813601</v>
+        <v>0.991682315281314</v>
       </c>
       <c r="G3">
-        <v>0.4786580191788909</v>
+        <v>0.4786580191782562</v>
       </c>
       <c r="H3">
-        <v>0.6321819358167948</v>
+        <v>0.6321819358172465</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -573,25 +579,25 @@
         <v>11</v>
       </c>
       <c r="B5">
-        <v>0.9445331155245272</v>
+        <v>0.9445331155262865</v>
       </c>
       <c r="C5">
-        <v>0.8035506396250885</v>
+        <v>0.8035506396251898</v>
       </c>
       <c r="D5">
-        <v>1.1754493978938485</v>
+        <v>1.1754493978958898</v>
       </c>
       <c r="E5">
-        <v>0.23981497051089873</v>
+        <v>0.2398149705100825</v>
       </c>
       <c r="F5">
-        <v>0.8016189913411198</v>
+        <v>0.8016189913412899</v>
       </c>
       <c r="G5">
-        <v>1.1782818592462612</v>
+        <v>1.1782818592482058</v>
       </c>
       <c r="H5">
-        <v>0.23868425741535604</v>
+        <v>0.23868425741458088</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -599,25 +605,25 @@
         <v>12</v>
       </c>
       <c r="B6">
-        <v>-0.011465758091658878</v>
+        <v>-0.011465758091649755</v>
       </c>
       <c r="C6">
-        <v>0.006429850139526603</v>
+        <v>0.006429850139526588</v>
       </c>
       <c r="D6">
-        <v>-1.7832076709182905</v>
+        <v>-1.7832076709168756</v>
       </c>
       <c r="E6">
-        <v>0.07455250424099913</v>
+        <v>0.07455250424122939</v>
       </c>
       <c r="F6">
-        <v>0.006283431512981876</v>
+        <v>0.0062834315129818765</v>
       </c>
       <c r="G6">
-        <v>-1.8247605735767252</v>
+        <v>-1.824760573575273</v>
       </c>
       <c r="H6">
-        <v>0.06803716791203995</v>
+        <v>0.06803716791225911</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -625,22 +631,22 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>-0.03394717514203955</v>
+        <v>-0.03394717514203287</v>
       </c>
       <c r="C7">
-        <v>0.0032947072297053377</v>
+        <v>0.0032947072297052414</v>
       </c>
       <c r="D7">
-        <v>-10.303548320156999</v>
+        <v>-10.303548320155272</v>
       </c>
       <c r="E7">
         <v>0.0</v>
       </c>
       <c r="F7">
-        <v>0.003293668386120358</v>
+        <v>0.0032936683861201676</v>
       </c>
       <c r="G7">
-        <v>-10.306798123664853</v>
+        <v>-10.30679812366342</v>
       </c>
       <c r="H7">
         <v>0.0</v>
@@ -651,25 +657,25 @@
         <v>14</v>
       </c>
       <c r="B8">
-        <v>-0.02068498987626741</v>
+        <v>-0.02068498987625425</v>
       </c>
       <c r="C8">
-        <v>0.006598906930824765</v>
+        <v>0.006598906930825106</v>
       </c>
       <c r="D8">
-        <v>-3.134608518214409</v>
+        <v>-3.1346085182122527</v>
       </c>
       <c r="E8">
-        <v>0.0017208359227158798</v>
+        <v>0.0017208359227285364</v>
       </c>
       <c r="F8">
-        <v>0.006571727803804811</v>
+        <v>0.006571727803805508</v>
       </c>
       <c r="G8">
-        <v>-3.1475725248832567</v>
+        <v>-3.1475725248809208</v>
       </c>
       <c r="H8">
-        <v>0.001646322596724259</v>
+        <v>0.0016463225967375816</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -677,25 +683,25 @@
         <v>15</v>
       </c>
       <c r="B9">
-        <v>-0.00884617192110412</v>
+        <v>-0.008846171921101768</v>
       </c>
       <c r="C9">
-        <v>0.0026240861017423835</v>
+        <v>0.0026240861017423327</v>
       </c>
       <c r="D9">
-        <v>-3.371143925205158</v>
+        <v>-3.3711439252043265</v>
       </c>
       <c r="E9">
-        <v>0.0007485673875702314</v>
+        <v>0.0007485673875724519</v>
       </c>
       <c r="F9">
-        <v>0.0025739209300067165</v>
+        <v>0.0025739209300066398</v>
       </c>
       <c r="G9">
-        <v>-3.436846803635509</v>
+        <v>-3.4368468036346975</v>
       </c>
       <c r="H9">
-        <v>0.0005885283773956473</v>
+        <v>0.0005885283773974237</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -703,25 +709,25 @@
         <v>16</v>
       </c>
       <c r="B10">
-        <v>-0.0036460770982343705</v>
+        <v>-0.0036460770982339797</v>
       </c>
       <c r="C10">
-        <v>0.001554502401701868</v>
+        <v>0.0015545024017018648</v>
       </c>
       <c r="D10">
-        <v>-2.345494670347661</v>
+        <v>-2.3454946703474144</v>
       </c>
       <c r="E10">
-        <v>0.01900185025568568</v>
+        <v>0.019001850255698338</v>
       </c>
       <c r="F10">
-        <v>0.0015685563312734171</v>
+        <v>0.0015685563312734102</v>
       </c>
       <c r="G10">
-        <v>-2.324479539268021</v>
+        <v>-2.3244795392677826</v>
       </c>
       <c r="H10">
-        <v>0.02009980693323188</v>
+        <v>0.020099806933244535</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -729,25 +735,25 @@
         <v>17</v>
       </c>
       <c r="B11">
-        <v>-0.011239353997987821</v>
+        <v>-0.011239353997999605</v>
       </c>
       <c r="C11">
-        <v>0.004385983456939217</v>
+        <v>0.004385983456939738</v>
       </c>
       <c r="D11">
-        <v>-2.5625618765628606</v>
+        <v>-2.5625618765652427</v>
       </c>
       <c r="E11">
-        <v>0.01039030713160849</v>
+        <v>0.010390307131537213</v>
       </c>
       <c r="F11">
-        <v>0.004408607980315356</v>
+        <v>0.004408607980316133</v>
       </c>
       <c r="G11">
-        <v>-2.549411072196047</v>
+        <v>-2.5494110721982706</v>
       </c>
       <c r="H11">
-        <v>0.010790502677975766</v>
+        <v>0.010790502677906932</v>
       </c>
     </row>
   </sheetData>
@@ -757,7 +763,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -765,7 +771,7 @@
         <v>18</v>
       </c>
       <c r="B1">
-        <v>-1025.756379460327</v>
+        <v>-1025.7563794603282</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -796,48 +802,56 @@
       <c r="A5" t="s">
         <v>22</v>
       </c>
-      <c r="B5">
-        <v>0.25056004524230957</v>
+      <c r="B5" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B6">
-        <v>9</v>
+        <v>0.8382189273834229</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B7">
-        <v>1000</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8">
-        <v>2069.512758920654</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B9">
-        <v>2113.682556431493</v>
+        <v>2069.5127589206563</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10">
-        <v>0.12392915222483869</v>
+        <v>2113.6825564314954</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11">
+        <v>0.12392915222483769</v>
       </c>
     </row>
   </sheetData>

</xml_diff>